<commit_message>
feat: flexible role rules, color-only roles, side-by-side export
- Lead and SME now require at least 2 each, with per-team counts differing by at most 1

- Result area and role config identify roles by color only; role panel uses three color swatches

- Export results as Team A names / blank separator / Team F names, names only

- Update tests, fixtures, README and rebuild MemberSplit.html
</commit_message>
<xml_diff>
--- a/test/fixtures/stress.xlsx
+++ b/test/fixtures/stress.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="N7" sheetId="1" r:id="rId1"/>
-    <sheet name="N8" sheetId="2" r:id="rId2"/>
-    <sheet name="N9" sheetId="3" r:id="rId3"/>
-    <sheet name="N10" sheetId="4" r:id="rId4"/>
-    <sheet name="N11" sheetId="5" r:id="rId5"/>
-    <sheet name="N50" sheetId="6" r:id="rId6"/>
+    <sheet name="N4-L2S2" sheetId="1" r:id="rId1"/>
+    <sheet name="N7-L2S5" sheetId="2" r:id="rId2"/>
+    <sheet name="N8-L3S2" sheetId="3" r:id="rId3"/>
+    <sheet name="N9-L4S3" sheetId="4" r:id="rId4"/>
+    <sheet name="N11-L5S4" sheetId="5" r:id="rId5"/>
+    <sheet name="N12-L3S9" sheetId="6" r:id="rId6"/>
+    <sheet name="N50-L7S15" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -402,6 +403,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B5"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Role</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Person 01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Team Lead</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Person 02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Team Lead</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Person 03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Person 04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -479,7 +535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
   <cols>
@@ -516,7 +572,7 @@
         <v>Person 03</v>
       </c>
       <c r="B4" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="5">
@@ -540,7 +596,7 @@
         <v>Person 06</v>
       </c>
       <c r="B7" t="str">
-        <v>SME</v>
+        <v>Member</v>
       </c>
     </row>
     <row r="8">
@@ -548,7 +604,7 @@
         <v>Person 07</v>
       </c>
       <c r="B8" t="str">
-        <v>SME</v>
+        <v>Member</v>
       </c>
     </row>
     <row r="9">
@@ -566,7 +622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B10"/>
   <cols>
@@ -603,7 +659,7 @@
         <v>Person 03</v>
       </c>
       <c r="B4" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="5">
@@ -611,7 +667,7 @@
         <v>Person 04</v>
       </c>
       <c r="B5" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="6">
@@ -657,109 +713,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Role</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Person 01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Team Lead</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Person 02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Team Lead</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Person 03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>SME</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Person 04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>SME</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Person 05</v>
-      </c>
-      <c r="B6" t="str">
-        <v>SME</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Person 06</v>
-      </c>
-      <c r="B7" t="str">
-        <v>SME</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Person 07</v>
-      </c>
-      <c r="B8" t="str">
-        <v>SME</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Person 08</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Member</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Person 09</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Member</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Person 10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Member</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -801,7 +754,7 @@
         <v>Person 03</v>
       </c>
       <c r="B4" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="5">
@@ -809,7 +762,7 @@
         <v>Person 04</v>
       </c>
       <c r="B5" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="6">
@@ -817,7 +770,7 @@
         <v>Person 05</v>
       </c>
       <c r="B6" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="7">
@@ -841,7 +794,7 @@
         <v>Person 08</v>
       </c>
       <c r="B9" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="10">
@@ -849,7 +802,7 @@
         <v>Person 09</v>
       </c>
       <c r="B10" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="11">
@@ -876,6 +829,125 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B13"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Role</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Person 01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Team Lead</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Person 02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Team Lead</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Person 03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Team Lead</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Person 04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Person 05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Person 06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Person 07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Person 08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Person 09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Person 10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Person 11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Person 12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>SME</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B51"/>
   <cols>
@@ -912,7 +984,7 @@
         <v>Person 03</v>
       </c>
       <c r="B4" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="5">
@@ -920,7 +992,7 @@
         <v>Person 04</v>
       </c>
       <c r="B5" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="6">
@@ -928,7 +1000,7 @@
         <v>Person 05</v>
       </c>
       <c r="B6" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="7">
@@ -936,7 +1008,7 @@
         <v>Person 06</v>
       </c>
       <c r="B7" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="8">
@@ -944,7 +1016,7 @@
         <v>Person 07</v>
       </c>
       <c r="B8" t="str">
-        <v>SME</v>
+        <v>Team Lead</v>
       </c>
     </row>
     <row r="9">
@@ -952,7 +1024,7 @@
         <v>Person 08</v>
       </c>
       <c r="B9" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="10">
@@ -960,7 +1032,7 @@
         <v>Person 09</v>
       </c>
       <c r="B10" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="11">
@@ -968,7 +1040,7 @@
         <v>Person 10</v>
       </c>
       <c r="B11" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="12">
@@ -976,7 +1048,7 @@
         <v>Person 11</v>
       </c>
       <c r="B12" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="13">
@@ -984,7 +1056,7 @@
         <v>Person 12</v>
       </c>
       <c r="B13" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="14">
@@ -992,7 +1064,7 @@
         <v>Person 13</v>
       </c>
       <c r="B14" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="15">
@@ -1000,7 +1072,7 @@
         <v>Person 14</v>
       </c>
       <c r="B15" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="16">
@@ -1008,7 +1080,7 @@
         <v>Person 15</v>
       </c>
       <c r="B16" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="17">
@@ -1016,7 +1088,7 @@
         <v>Person 16</v>
       </c>
       <c r="B17" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="18">
@@ -1024,7 +1096,7 @@
         <v>Person 17</v>
       </c>
       <c r="B18" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="19">
@@ -1032,7 +1104,7 @@
         <v>Person 18</v>
       </c>
       <c r="B19" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="20">
@@ -1040,7 +1112,7 @@
         <v>Person 19</v>
       </c>
       <c r="B20" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="21">
@@ -1048,7 +1120,7 @@
         <v>Person 20</v>
       </c>
       <c r="B21" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="22">
@@ -1056,7 +1128,7 @@
         <v>Person 21</v>
       </c>
       <c r="B22" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="23">
@@ -1064,7 +1136,7 @@
         <v>Person 22</v>
       </c>
       <c r="B23" t="str">
-        <v>Member</v>
+        <v>SME</v>
       </c>
     </row>
     <row r="24">

</xml_diff>